<commit_message>
Querying using AMC DOI
</commit_message>
<xml_diff>
--- a/brown_validation_papers_with_text.xlsx
+++ b/brown_validation_papers_with_text.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="330">
   <si>
     <t>paper</t>
   </si>
@@ -1001,27 +1001,6 @@
   </si>
   <si>
     <t>pmid</t>
-  </si>
-  <si>
-    <t>Abstract
-Phosphoinositide 3-kinase (PI3K) is deregulated in a wide variety of human tumors and triggers activation of protein kinase B (PKB/Akt) and mammalian target of rapamycin (mTOR). Here we describe the preclinical characterization of compound 1 (PQR309, bimiralisib), a potent 4,6-dimorpholino-1,3,5-triazine-based pan-class I PI3K inhibitor, which targets mTOR kinase in a balanced fashion at higher concentrations. No off-target interactions were detected for 1 in a wide panel of protein kinase, enzyme, and receptor ligand assays. Moreover, 1 did not bind tubulin, which was observed for the structurally related 4 (BKM120, buparlisib). Compound 1 is orally available, crosses the blood−brain barrier, and displayed favorable pharmacokinetic parameters in mice, rats, and dogs. Compound 1 demonstrated efficiency in inhibiting proliferation in tumor cell lines and a rat xenograft model. This, together with the compound’s safety profile, identifies 1 as a clinical candidate with a broad application range in oncology, including treatment of brain tumors or CNS metastasis. Compound 1 is currently in phase II clinical trials for advanced solid tumors and refractory lymphoma.
-Introduction
-Phosphoinositide 3-kinases (PI3Ks) are lipid kinases that play a central role in the control of cancer cell growth, proliferation, and metastasis. 1 – 3 The PI3K family is divided into three classes according to sequence homology and substrate specificity: so-called class I PI3Ks are activated downstream of cell surface receptors, including receptor protein tyrosine kinases (RTKs), immunoglobulin receptors, and G-protein-coupled receptors (GPCRs). Class IA PI3Ks consist of the catalytic subunits p110 α , p110 β , and p110 δ . These interact with dedicated phosphorylated tyrosine motifs on growth factor receptors or their substrates via two src-homology 2 (SH2) domains present in their tightly associated p85 regulatory subunits. The class IB PI3K γ operates downstream of GPCRs and is composed of a catalytic subunit p110 γ and an adapter subunit, which is either p84 or p101. 4
-Class I PI3Ks phosphorylate phosphatidylinositol (4,5)-bisphosphate [PtdIns(4,5) P 2 ] to yield phosphatidylinositol (3,4,5)-trisphosphate [PtdIns(3,4,5) P 3 ]. PtdIns(3,4,5) P 3 , produced at the inner leaflet of the plasma membrane, provides a docking site for effector proteins with pleckstrin-homology (PH) domains. The serine/threonine kinases phosphoinositide-dependent kinase 1 (PDK-1) and protein kinase B (PKB/Akt) contain a PH domain and are thus activated by PI3K and relay the activation of the mammalian target of rapamycin complex 1 (mTORC1). In tumor cells, hyperactivation of the PI3K/mTOR pathway can occur on multiple levels, including mutation or overexpression of cell surface receptors such as HER2, 5 oncogenes, the protein tyrosine phosphatase non-receptor 12 (PTPN12), 6 or the presence of activating hotspot mutations in PIK3CA (encoding the catalytic PI3K α subunit p110 α ). 7 Other key regulators of the PI3K pathway include the lipid phosphatase PTEN, hydrolyzing PtdIns(3,4,5) P 3 back to PtdIns(4,5) P 2 , 2 , 8 and the inositol polyphosphate 4-phosphatase type II (INPP4B) 9 degrading PtdIns(3,4) P 2 . Loss of either lipid phosphatase activities or gain of function mutations at the level of PI3K, and aberrations up- and downstream in the pathway can thus lead to the constitutive activation of PI3K, PKB/Akt, and mTOR.
-Besides promotion of tumor cell growth and angiogenesis, an overactivated PI3K/mTOR pathway has been associated with resistance to other cancer treatments, e.g., receptor tyrosine kinase inhibitors. PI3K inactivating agents are currently in various clinical trials as monotherapy or in combination with other drugs. 2 , 3 , 10
-In our search for the development of a dual pan-PI3K/mTOR inhibitor, we focused on dimorpholino substituted compounds with a triazine core, as their symmetry supports rapid access to a compound library with various aryl substituents. Furthermore, our goal was to develop brain-penetrable compounds to allow for the treatment of brain metastasis and brain tumors. Here we describe a SAR study around the aryl moiety at the C2-position of bismorpholino-triazines, which led to the identification of 1 (PQR309, bimiralisib), 11 a clinical candidate and brain penetrable pan-PI3K/mTOR inhibitor.
-Results and Discussion
-Compound 1 evolved as the lead compound of a series of dimorpholinotriazine based compounds and is currently tested in phase II clinical trials ( clinicaltrials.gov ). Initially inspired by 2-(2-difluoromethylbenzimidazol-1-yl)-4,6-dimorpholino-1,3,5-triazine (ZSTK474), 12 a pan PI3K inhibitor with a triazine core, development of 1 aimed to (i) maximize compound solubility and bioavailability, (ii) achieve blood–brain barrier penetration, (iii) avoid microtubule interactions as observed for 4 (BKM120, buparlisib), 11 , 13 and (iv) introduce moderate mTOR inhibition. The rationale for PI3K/mTOR dual activity was based on the observation that persistent mTOR signaling was reported to confer resistance to PI3K inhibition, 14 while selective targeting of the mTOR complex 1 (TORC1) initiates positive feedback leading to PI3K hyperactivation. 15 To avoid this, we selected for compounds with a higher potency for PI3K than mTOR kinase. Moreover, drugs targeting both PI3K and mTOR have been shown early on to be more effective in tumors with multiple pathway activation such as melanoma 16 , 17 and to potentially support drug combinations. 18
-A number of clinically advanced PI3K inhibitors with a pyrimidine, triazine, or fused pyrimidine core contain at least one morpholine moiety. This morpholine was demonstrated to be a crucial feature for PI3K binding, as the morpholine oxygen atom forms a hydrogen bond interaction with the hinge region backbone NH of the amino acid residue Val851 in PI3K α (Val882 in PI3K γ , and Val2240 in mTOR). Structurally related compounds, which display distinct PI3K and mTOR kinase inhibitory profiles ( Table 1 ), are shown in Figure 1 : 1 , 4 , 19 and 6 (GDC-0980, apitolisib/RG7422)20 target PI3K and mTOR kinase with some preference for PI3K α , while 3 (PIK-587, gedatolisib/PF-05212384) 21 is a potent dual PI3K/mTOR inhibitor and 5 (GDC-0941, pictilisib) 22 targets PI3K.
-Table 1. Affinity of Triazine and Pyrimidine Core-Containing Molecules to PI3K and PI3K-Related Kinases. binding constant K d [nM] a compd PI3K α PI3K β PI3K γ PI3K δ mTOR PI3KC2 β VPS34 PI4KC β DNAPK mTOR/PI3K α 1 1.5 11 25 25 12 820 230 40000 1600 8.0 2 1.2 3.5 11 3.5 61 540 130 27000 &gt;30000 51 3 1.0 3.5 24 76 0.94 0.46 5100 &gt;30000 &gt;30000 0.94 4 3.5 36 130 260 19 2100 200 40000 1800 5.4 5 0.76 2.1 7.7 3.3 48 40 nd 40000 1300 63 6 0.62 3.8 2.6 3.3 3.3 580 250 &gt;30000 9800 5.3 IC 50 , kinase assay [nM] b compd PI3K α PI3K β PI3K γ PI3K δ mTOR α 542K/545K/1047R c VPS34 DNAPK mTOR/PI3K α 1 33 661 708 451 89 63/136/36 8486 8567 2.6 4 45 607 778 110 94 111/216/87 2581 6917 13 Open in a new tab a Dissociation constants ( K d ) were determined using ScanMax technology (DiscoveRx) 26 with 11-point 3-fold serial dilutions of the indicated compounds. K d is the mean value from experiments performed in duplicate and calculated from standard dose–response curves using the Hill equation depicted in Experimental Section ( n ≥ 2). A TreeSpot representation of a full kinase panel and kinase residual binding values are shown in Supporting Information Figure S1 and Table S2 for all above compounds except compound 2 . b Prokinase activity assays of the indicated enzymes and PI3K α mutants. c Inhibition of PI3K α E542K, E545K, and H2047R mutant activities are indicated. For these values, the wild type PI3K α reference IC 50 values were 122 nM for 1 and 142 nM for 4 .
-Figure 1. Open in a new tab Structure of triazine core PI3K inhibitors 1 , reference compound 2 , reported clinical candidate 3 , and pyrimidine or fused pyrimidine core containing molecules 4 , 5 , and 6 .
-The above compounds are substituted with various aryl moieties (e.g., indazole, pyrimidine, pyridine, benzoimidazole, or aniline), which are situated in the PI3K’s ATP-binding site toward the affinity binding pocket. The primary amine of 4 11 , 19 and 6 20 interacts via hydrogen bonding with the carboxyl groups of the amino acid residues Asp841 and Asp836 in PI3K γ . For 3 it has been proposed that the urea-NH groups form hydrogen bonds with Asp810 and the urea oxygen engages the wortmannin-reactive Lys802 23 , 24 in PI3K α . 25 Finally, 5 exploits its indazole N-NH atoms to form hydrogen bonds with Tyr867 and Asp841 in PI3K γ . As illustrated by the exchange of the aryl moiety from 4-(trifluoromethyl)pyridin-2-amine in 1 to 4-(trifluoromethyl)pyrimidin-2-amine in compound 2 , the aryl substitution can be used to fine-tune PI3K vs mTOR activity.
-Chemistry To achieve a balanced PI3K and mTOR inhibition and to adjust physicochemical properties, a library of 4,6-dimorpholino-1,3,5-triazines substituted with various C-2-aryl moieties was prepared from 4,4′-(6-chloro-1,3,5-triazine-2,4-diyl)dimorpholine ( 7 , Scheme 1 ). The chlorine was displaced by aniline or heteroaryl moieties using Suzuki cross-coupling reactions with boronic acid pinacol esters. The desired products were obtained in moderate to good yield (11–86%) depending on the used boronic acid pinacol ester derivative. Moreover, compound 1 was transformed by acetylation and diazotization followed by bromination and Sandmeyer reaction in order to obtain derivatives bearing different substituents at the C-2 pyridine ( 17 – 21 ). All final compounds were analyzed for purity by analytical HPLC (&gt;95%). Scheme 1. Synthesis of C-2-Aryl-Substituted 4,6-Dimorpholino-1,3,5-triazine Analogs a . Open in a new tab a . a Reagents and conditions: (i) ArBpin, XPhosPdG2 (cat.), K 3 PO 4 , dioxane/H 2 O, 95 °C, 2–16 h, then HCl (aq), 60 °C, 2–8 h; (ii) ArBpin, Pd(dppf)Cl 2 (cat.), Na 2 CO 3 , 1,2-dimethoxyethane/H 2 O, 90 °C, 16 h; (iii) ArBpin, XPhosPdG2 (cat.), K 3 PO 4 , dioxane/H 2 O, 95 °C, 2 h; (iv) AcCl, K 2 CO 3 , CH 2 Cl 2 , 0 °C → rt, 3.5 h; (v) HCl (conc), NaNO 2 , 0 °C → rt, 1 h, then CuCl, rt, 1 h; (vi) isopentyl nitrite, CH 2 Br 2 , rt, 5 min, then (CH 3 ) 3 SiBr, rt, 1 h; (vii) CH 3 ONH 2 ·HCl, NaHCO 3 , DMSO, 100 °C, 6 h. b Compound 1 was prepared according to the procedure recently reported. 11 ArBpin: boronic acid pinacol ester (the amino group was protected in certain cases). We have recently reported an optimized synthetic route to compound 1 . 11 This strategy allowed for rapid access to large quantities of 1 starting from cyanuric chloride (81% yield) for preclinical and clinical development.
-Determination of Cellular Potency and PI3K vs mTOR Kinase Activities In the following studies, the role of the aryl moiety was investigated systematically for enzymatic activity and selectivity for class IA PI3K versus mTOR ( Table 2 ). A first series of compounds including variations of nitrogen atoms number and position was prepared to study the effect of the polarity of the aryl group ( 9 – 12 ). Interestingly, 10 and 11 substituted with 2-aminopyridine and 2-aminopyrimidine, respectively, were both found to be active in cellular and enzymatic assays. The calculated PSA (polar surface area) value for the pyridine-substituted 10 (PSA = 103) was slightly lower as compared to pyrimidine 11 (PSA = 115), predicting a better brain penetration for 10 . Therefore, pyridines were substituted with lipophilic substituents such as methyl and trifluoromethyl at pyridine C3 and C4 positions to generate compounds 13 – 15 . Introduction of a C4-trifluoromethyl group significantly increased cellular potency and enzymatic targeting: compared with 13 , 1 showed excellent cellular activities, good potency in vitro ( K i for PI3K α of 17 nM), targeted mutated forms of the catalytic PI3K α subunit, and displayed the desired selectivity profile targeting PI3K α &gt;mTOR ( K i ratio of mTOR/p110 α of ~3.6 [~8.0 from KINOMEscan; see Table 1 ]). On the contrary, introduction of a lipophilic substituent at the C3-position (methyl in 14 and trifluoromethyl in 15 ) diminished binding to PI3K α as well as to mTOR. Table 2. Direction of PI3K/mTOR Selectivity with Aromatic Substituents for Dimorpholinotriazine. Cmpd Cellular IC 50 [nM] a , b in vitro K i [nM] c Growth Growth mTOR/PI3Kα clogP d PSA d pPKB/Akt pS6 PI3Kα mTOR A2058 SKOV3 9 1744 1282 12630 8504 1513 396 0.26 2.45 89.6 10 367 415 3819 742 123 110 0.89 2.23 103 11 330 415 2161 270 46 106 2.34 1.39 115 12 1283 817 9083 4428 911 185 0.20 1.31 115 13 401 939 9113 1504 61 609 10.00 2.69 102 1 139 205 2333 237 17 62 3.60 3.11 102 14 1620 1105 14210 6221 1205 241 0.20 2.69 102 15 2370 1638 &gt;20000 9213 4.3e6 284 6.5e-5 3.11 102 16 169 831 2934 342 13 224 17.60 1.56 115 2 85 312 1636 73 8.1 203 25.10 2.67 115 20 3303 5588 19200 4545 689 2539 3.70 3.09 97.8 17 208 729 14480 11500 9.7 1213 125.00 3.22 105 18 1.3e5 1.7e7 &gt;20000 &gt;20000 2299 n.d. – 3.61 96.7 19 51971 1.1e6 4347 14050 32833 1.1e5 3.22 4.08 76.5 21 1.5e5 n.d. 3033 3654 n.d. 6.6e5 – 4.38 76.5 Open in a new tab a Cellular phosphorylation of PKB/Akt on Ser473 and ribosomal S6 on Ser235/236 were analyzed in inhibitor treated A2058 melanoma cells using in-cell Western detection. Each experiment was performed in triplicate or as a multiple of n = 3. b IC 50 values of A2058 or SKOV3 cell proliferation were determined from 10-point 2-fold serial dilutions ( n = 3). c Compounds were tested in a time-resolved FRET (TR) assay (LanthaScreen), and inhibitor K i values were calculated for PI3K α and mTOR as described in Experimental Section . The mTOR/PI3K α column depicts the ratio of compound-specific mTOR K i over the K i for PI3K α . Each experiment was performed at least twice or as a multiple of n = 2. d Marvin/JChem 16.10.17 was used for calculation of log P (partition coefficient) and PSA (polar surface area) values. While compound 11 , bearing an unsubstituted 2-amino-pyrimidine, turned out to be a balanced inhibitor for PI3K α and for mTOR in vitro, ( K i (mTOR)/ K i (PI3K α ) ≈ 2.3), a substitution at the pyrimidine C4-position with methyl ( 16 ) or trifluoromethyl ( 2 ) enhanced cellular and in vitro activity toward PI3K α and diminished affinity for mTOR, raising the mTOR/PI3K α K i ratio to ~16–25. Modifications at the C2-pyridine position of the most potent compound 1 were also investigated ( 17 – 21 ). These changes alter both the steric and the electronic properties of the amine group and are likely to affect hydrogen bond interactions with the aspartate carboxy groups in the affinity binding pocket (Asp841 and Asp836 in PI3K γ ). Hydroxylamine and amide moieties replacing primary amine functionality in 1 impaired binding to mTOR ( K i &gt; 1 μ M), and replacing the primary amine moiety by a hydroxylamine, amide, hydroxy, or halide decreased cellular potency considerably. Compound 17 retained its affinity for PI3K α in spite of an amide extension, likely due to a hydrogen bond of the amide carbonyl with Lys802 (Lys833 in PI3K γ : in analogy to compound 26 in ref 27 [see also PDB code 3IBE]). The SAR study depicted above led to the identification of two potent compounds 1 and 2 , both substituted with a trifluoromethyl group on their aryl moiety. Both of them showed excellent potency for PI3K α , cellular activity profiles, and a calculated log P value of ~3. Compound 1 was investigated in more detail, as it displayed a mTOR/PI3K α K i selectivity ratio in the range of 3–8, while 2 had reduced impact on mTOR ( Tables 1 and 2 ). An additional point in favor of compound 1 was a lower calculated PSA value of 102 as compared to 115 for 2 , predicting a better brain penetration for 1 .
-Binding Mode of Compound 1 to PI3K and mTOR Kinase Binding of compound 1 to the PI3K γ catalytic subunit p110 γ ATP-binding site was confirmed by a 2.7 Å complex crystal structure and identified key interactions of 1 with residues of p110 γ . As reported for other morpholino-substituted PI3K inhibitors including compound 4 , 11 , 19 one morpholine of 1 forms a hydrogen bridge with the backbone amide of Val882, a well-known and crucial interaction. 28 The compound 1 /PI3K γ complex crystal structure (PDB code 5OQ4; Table S1 in Supporting Information) also showed that the amino group of the 2-amino-4-(trifluoromethyl)pyridine moiety forms H-bonds with Asp836, Asp841, and Asp964 ( Figure 2A ). Given the high homology of class I PI3K catalytic pockets and the nanomolar in vitro dissociation constants of 1 for all class I PI3Ks ( Table 1 ), an identical binding mode for all PI3K isoforms can be assumed. Besides the high affinity for class I PI3K isoforms (highest affinity for PI3K α ), compound 1 ’s affinity for mTOR kinase is comparable to PI3K β , PI3K γ , and PI3K δ ( Table 1 ). Figure 2. Open in a new tab Interactions of 1 with the ATP-binding site of PI3K γ catalytic subunit p110 γ and mTOR kinase. (A) Crystal structure of 1 in PI3K γ with a resolution of 2.7 Å (PDB code 5OQ4; Table S1 ). Compound 1 interacts with the hinge valine V882 in PI3K γ , and its heteroaryl amine function forms hydrogen bonds with the carboxyl groups of aspartates D836, D841, and D964. (B) Overlay of the compound 1 /PI3K γ complex coordinates with the compound 4 /PI3K γ data from PDB accession code 3SD5. 19 The pyrimidine core nitrogen atom positions are corrected for the orientation as proposed in ref 11 (* denotes the position of C–H in compound 4 ); the two molecules are oriented exactly as in (A). (C) The coordinates of a mTOR kinase/PI103 complex resolved to 3.6 Å (PDB code 4JT6; docked, yellow) and mTOR at a resolution of 3.2 Å (PDB code 4JSN; relaxed, turquoise) were used to dock 1 into the ATP-binding site of mTOR kinase. The yellow structure represents the results of a manual predocking process (docked) where PI103 was replaced by 1 with subsequent energy minimization. The turquoise structure represents the best fit of dynamic docking procedures to 4JSN (relaxed starting conditions). Dotted lines indicate proposed H-bond interactions. The current compound 1 /PI3K γ X-ray crystal structure combined with our previous structural studies on 4 and an asymmetrically substituted triazine (PIKiN3, PDB code 5JHB) 11 underlines the importance of Asp836, Asp841, and Asp964 and associated structured water molecules for the binding of this compound class. Changes in the basicity of the amino-heteroaryl (2-amino-4-(trifluoromethyl)pyridine in 1 are therefore expected to affect the affinity for PI3K, as it was the case for 2-aminopyrimidine 2 . The situation in the mTOR catalytic pocket is less well-defined: (i) modeling compound 1 /mTOR interactions starting with a predocked inhibitor generate an interaction pattern similar to PI3K, where carboxyl groups of Asp2357, Glu2190, and Asp2195 are at a distance of 3.5–4 Å from the heteroaryl amino group and could execute hydrogen bonding; (ii) starting with less constraints, the inhibitor is slightly displaced by docking procedures, and the sole residue in hydrogen bonding distance remains Glu2190. Although less conventional, the latter structure offers some explanation for the differential effects of heteroaryl modifications for PI3K and mTOR affinity shown in Table 2 .
-On- and Off-Target Activities In line with its activities against PI3K and mTOR, compound 1 induced a G1 cell cycle arrest in A2058 melanoma cells (mutated B-Raf, loss of PTEN) and SKOV3 cells (PI3K α mutated at H1047R), which have both constitutively activated PI3K/mTOR signaling pathways. In contrast, compound 4 triggered a mitotic arrest and cells accumulated in G2/M or subG1 ( Figure 3 ), which is in agreement with the reported binding of 4 to the colchicine-binding site of tubulin. 11 In spite of compound 4’s off-target effect, the compound attenuated PI3K and mTOR signaling as determined by protein kinase B (PKB/Akt) phosphorylation on Ser473 and Thr308 and by S6 kinase (S6K, Thr389) and S6 phosphorylation on Ser235 and Ser236. Here, 4 closely matched the action of 1 , 5 , 6 , 3 , and 2 , while rapamycin by its specific action on TORC1 triggered an upregulation of PI3K activity, which is in agreement with earlier observations. 29 Figure 3. Open in a new tab Action of indicated compounds on cell cycle and PI3K and mTOR signaling. Cell cycle distribution of A2058 (A) and SKOV3 (B) cells after 24 h exposure to 5 μ M (A) or 2 μ M (B) of indicated drugs ( 1 , green; 4 , red) or DMSO. After drug exposure cells were collected, fixed, permeabilized and the DNA was stained using propidium iodide. Cell cycle profiles were acquired by fluorescence activated cell sorting. Left panels: Examples of cell cycle histograms. Right panels: Quantification of cells in cell cycle phases G1, S, G2/M, and sub-G1 (as % of total, n = 9, mean ± SD, one way ANOVA test with Dunnett’s multiple comparison test for each cell cycle phase related to DMSO; ns, not significant, (**) p &gt; 0.0021, (****) p &gt; 0.0001). (C, D) A2058 or SKOV3 cells were exposed to 1 μ M drug (rapamycin 100 nM) for 1 h, subsequently lysed, and the denatured lysates subjected to SDS–PAGE, Western blotting, and immune detection. (C) Detection of total and phosphorylated (pT308 and pS473) PKB/Akt, and α -tubulin (left, A2058; right, SKOV3). Top: Quantification of phospho-PKB/Akt levels related to DMSO control (blue, pT308; red, pS473; n = 3, mean ± SEM). (D) Detection of total and phosphorylated (pS235/236) ribosomal protein S6 and of total and phosphorylated (S6K T389) S6 kinase (left, A2058; right, SKOV3). Top: Quantification of phospho-protein levels, related to DMSO control (blue, phospho S6; red, phospho S6K; n = 3, mean ± SEM). To validate the specificity of 1 , the compound was tested in a KINOMEScan panel for interactions with a wide range of protein (&gt;400) and lipid kinases in parallel with 4 , 5 , 6 , and 3 . At 10 μ M concentration 1 , 4 , 5 , and 3 did show negligible interference with protein kinase activities ( Figure S1, Table S2 ), while the dual PI3K/mTOR kinase inhibitor 6 displayed multiple hits. Compound 1 reached excellent selectivity scores of S (35) = 0.025, S (10) = 0.018, as calculated according to ref 30 . The impact of compound 1 on cell proliferation was analyzed in four independent human tumor cell line collections of different tissue origin (NCI60; 31 NTRC, The Netherlands; Horizon Discoveries, U.K.; Clovis, U.K.; 135 different cell lines in total). Combined across the four cell panels the mean half-maximal growth inhibition (GI 50 ) was reached at ~0.7 μ M (median: ~0.5 μ M) for 1 as depicted in Figure 4 . Figure 4. Open in a new tab Cell proliferation in response to 1 represented as a waterfall blot. Concentrations of half-maximal growth inhibition (GI 50 for 1 were obtained from dose–response growth curves derived from 4 different tumor cell line panels (a total of 135 cell lines; if a cell line was contained in several panels, its GI 50 was averaged). Individual GI 50 of a cell line was related to the mean GI 50 of all cells lines, and cell lines were sorted by lowest to highest sensitivity for 1 from left to right. Individual cell lines and values for the four cell panels are given in Table S3 . We have previously compared IC 50 -independent parameters such as Hill slopes of proliferation inhibition curves and dose-dependent induction of nuclear condensation and histone H3 phosphorylation in a 44 cell line panel treated with either 1 , 4 , 5 , or 6 , which showed a coclustering of the PI3K inhibitors 1 , 5 , and 6 and grouped 4 with inhibitors of mitosis such as colchicine, nocodazole, and MTD147, a microtubule-binder derived from 4 , 11 corroborating that 1 is free of the microtubule-binding off-target action of 4 . To evaluate other off-target effects, compound 1 was tested at 10 μ M in a CEREP BioPrint panel, where no or only very weak competition with radioligands for cell surface and nuclear receptors, membrane channels, transporters ( Table S4 ) and enzyme activities of kinases, proteases, and phosphodiesterases ( Table S5 ) were detected. Altogether, 1 qualifies as a specific pan-class I PI3K inhibitor without predicted off-target effects.
-Pharmacological Parameters of Compound 1 Before translation of the in vitro and cellular activities to in vivo tumor models, pharmacological properties and metabolic stability of 1 were assessed. Compound 1 showed little clearance when exposed to rat, dog, and human liver microsomes, with a quicker turnover of 1 in mouse liver microsomes, where 40% of the compound was eliminated within 30 min ( Table 3 ). Stability in microsome assays was matched with clearance and half-live measurements in human, cynomolgus monkey, rat, dog, and mouse hepatocyte cultures, where 1 showed a low clearance in all species except for mouse. In the presence of human hepatocytes, the half-life of compound 1 was 9.4 h and ~45 min in mouse hepatocytes ( Table 4 ). Table 3. Stability in Liver Microsomes of Compound 1. % remaining in liver microsomes a compd human rat dog mouse 1 84.6 ± 2.2 99.9 ± 0.5 92.4 ± 1.6 60.7 ± 4.6 7-EC b 7.45 ± 0.8 28.5 ± 3.1 1.8 ± 1.0 1.5 ± 0.03 propranolol b 54.8 ± 6.7 2.9 ± 0.1 30.1 ± 2.6 6.8 ± 0.9 Open in a new tab a Percentage of compound remaining after 30 min (mean ± SD, n = 2). b Assay reference compounds. 7-EC: 7-ethoxycoumarin. Table 4. Stability of Compound 1 in Hepatocyte Cultures a . compd parameter human monkey rat dog mouse 1 CL int b 2.5 ± 0.4 3.5 ± 0.1 1.9 ± 0.1 2.4 ± 0.1 30.3 ± 0.1 t 1/2 [min] 562.6 ± 95.5 396.4 ± 16.0 731.7 ± 54.5 577.6 ± 0.1 45.7 ± 0.2 7-EC c CL int b 37.8 ± 0.8 61.1 ± 3.5 16.0 ± 0.8 151.4 ± 2.8 180.3 ± 0.1 t 1/2 [min] 36.7 ± 0.8 22.7 ± 1.3 86.8 ± 4.6 9.2 ± 0.2 7.7 ± 0.1 7-HC c CL int b 98.2 ± 5.1 92.5 ± 3.5 192.8 ± 14.4 178.3 ± 0.7 188.1 ± 8.6 t 1/2 [min] 14.1 ± 0.7 15.0 ± 0.6 7.2 ± 0.5 7.8 ± 0.1 7.4 ± 0.3 Open in a new tab a Results are expressed as mean ± SD, n = 2. b CL int [( μ L/min)/10 6 cells]. c Assay reference compounds: 7-EC, 7-ethoxycoumarin; 7-HC, 7-hydroxycoumarin. Subsequently, in vivo pharmacological parameters were determined in female CD-1 mice, female Sprague-Dawley rats, and male Beagle dogs to assess optimal dosing schedules for efficacy studies. Compound 1 was delivered by either a single intravenous (5 mg/kg) bolus or a single oral application (10 mg/kg). Drug levels in extracts of plasma, brain, and liver were determined by LC–MS/MS ( Figure 5 ; PK parameters are summarized in Table 5 ). In female mice, plasma concentrations of 1 depended on the drug administration route, resulting in half-lives of approximately 13–36 min for po administration vs 9–10 min for iv administration. The fact that oral administration yielded similar concentrations of 1 in brain and plasma samples illustrates that compound 1 readily passes the blood–brain barrier. In mice, both po and iv application routes showed a rapid drop below 200 ng/mL (~0.5 μ M, Figure 5A ) of 1 within &lt;1 h (iv) to &lt;2 h (po) after administration, which reflects the time point when the drug reaches the median GI 50 determined in tumor cell lines. Figure 5. Open in a new tab PK/PD assessment of 1 in mice, rats, and dogs: time course of 1 abundance in vivo. Compound 1 was administered in all species as single dose either per os (po, 10 mg/kg) or via intravenous injection (iv, 5 mg/kg). At indicated time-points 1 was extracted from tissue and its abundance determined using HPLC/MS–MS. (A) Levels of 1 in CD1-mice tissue. Right graph: Zoomed view on early time points, indicated in left graph by dashed square ( n = 3, mean ± SD). (B) Concentrations of 1 in tissues from Sprague-Dawly rats. Right graph: Zoomed view on early time points, indicated in left graph by dashed square ( n = 3, mean ± SD). (C) Plasma levels of 1 in male Beagle dogs. Panels on the right: zoomed in to dotted line boxes to visualize early time points ( n = 3, mean ± SD). Table 5. PK Analysis of 1 in Plasma of Mice, Rats, and Dogs a . parameter female CD-1 mouse female Sprague-Dawley rats male Beagle dog route iv po iv po iv po dose [mg/kg] 5 10 5 10 5 10 C max [ng/mL] 3084 ± 379 1514 ± 334 3047 ± 557 4028 ± 1179 8760 583 T max [min] 5 15 5 15 5 120−240 t 1/2 [h] 0.15−0.33 0.22−0.60 5.6−8.2 5.6 7.6 8.6 AUC [h·ng/mL] 1583 AUC 0−8h 2151 AUC 0−8h 13974 AUC 0.25−12h 15313 AUC 0.25−12h 12500 AUC 0.25−24h 6395 AUC 0.017−24h Cl [mL h −1 kg −1 ] 3180 266 411 BA [%] 68 55 23 Open in a new tab a iv, intravenous (5 mg/kg); po, per os (10 mg/kg); C max , maximal concentration; T max , time of maximal concentration in hours; t 1/2 , half-life elimination in hours; AUC, area under curve; Cl, clearance; BA, bioavailability. n = 3, mean ± SD for each time point, species, and route. In female rats a single oral dose (10 mg/kg) achieved similar drug levels as a single intravenous injection (5 mg/kg) with regard to C max (see Table 5 ). The half-life of 5–8 h and an AUC 0.25–12 of around 14 000 h·ng/mL contributed to an excellent oral bioavailability of 1 (&gt;50%). Twenty-four hours after po administration, plasma levels of 1 were still &gt;2 μ M (800–1000 ng/mL). Moreover, after 1–2 h exposure to 1 , drug levels in rat brain samples were comparable to plasma levels ( Figure 5B ), confirming rapid access of 1 to the brain. Male Beagle dogs, exposed to 1 at 10 mg/kg po, showed maximal drug plasma concentrations C max of 583 ng/mL (approximately 1.5 μ M) after 60–90 min and a half-life of &gt;7 h, which results in drug levels of approximately 0.38 μ M (150 ng/mL) after 24 h. Intravenous delivery of 5 mg/kg of 1 resulted in high immediate concentrations (&gt;7000 ng/mL after 1 min), and plasma levels decreased within 8 h to similar concentrations as observed for oral dosing ( Figure 4C ). The oral bioavailability in male Beagle dogs was estimated to be 23%. In vitro and in vivo toxicokinetic parameters were assessed and are summarized in Table S6 . In rodents and Beagle dogs, compound 1 showed moderate but reversible target organ toxicity, which is expected for this drug class and mechanism of action. Altogether the PK studies in the three models show rapid absorption of 1 and good oral bioavailability. Except for mice with a rapid clearance of 1 , the late phase concentrations of 1 in rats and dogs are in the expected range of predicted efficacy, independent of the administration route, and are already reached after a single dose. The collected parameters are compatible with oral dosing in humans once daily (QD). Altogether, compound 1 displays a superior solubility ( Table S7 ) as compared with compound 2 , is orally bioavailable and brain penetrable, and does not display a microtubule-binding off-target effect like compound 4 . 11
-Efficacy Models Due to the short half-live of compound 1 in mice, a PC3 xenograft model in nude rats was used to assess the antiproliferative effects of 1 in vivo. Rats were injected with 2 × 10 7 human PC3 prostate cancer cells into one flank and randomized after 16 days. From day 17 the control group received vehicle once daily. Compound 1 was orally administered at 5 mg/kg, 10 mg/kg (both daily, QD), or 15 mg/kg [5 consecutive days, 2 days off drug (QD × 5, 2 days off)] for 28 days to match the timelines of regulatory toxicology studies. A vinorelbine-treated group (2.5 mg/kg iv weekly) was included as a “standard of care” control, with best treated-to-control ratios ( T / C ) of 17%. Treatment with 1 led to significant tumor size reductions: tumor growth was inhibited dose-dependently (best T / C of 31–12%, Figure 6A ). Compound 1 was best tolerated at 5 mg/kg without significant body weight changes ( Figure 6B ). At 10 mg/kg, 1 caused a reduction of body weight, which accumulated to a reduction of 15% after 28 days of treatment. Similarly, 15 mg/kg of 1 led to body weight loss after 5 days of treatment, which was reversible during the recovery period. After 28 days of drug exposure (day 44 of the experiment), animals with body weight loss fully recovered within a treatment-free period (days 45–50) without overt signs of tumor cell proliferation. In a subsequent treatment period tumor growth remained inhibited and body weight loss was only observed in the 15 mg/kg group. Figure 6. Open in a new tab Efficacy model for antitumor activity of 1 in PC3 xenografts in nude rats. (A) Tumor volume: Indicated amounts of 1 (po, daily) or vinorelbine (iv, weekly) were given from day 17 to day 44 and from day 51 to day 58 after tumor inoculation (see Experimental Section ; n = 4–8, mean ± SEM). (B) Body weight changes in nude rats (treated as in (A), n = 4–8, mean ± SEM). (C) Time course of 1 abundance in nude rats. Compound 1 was administered as single dose per os (po, 15 mg/kg). At indicated time points 1 was extracted from tissue and</t>
   </si>
   <si>
     <t>Abstract
@@ -1454,16 +1433,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1479,7 +1450,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1487,30 +1458,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1809,61 +1762,61 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:19">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2075,8 +2028,8 @@
       <c r="Q5" t="b">
         <v>1</v>
       </c>
-      <c r="S5" t="s">
-        <v>329</v>
+      <c r="R5" t="s">
+        <v>328</v>
       </c>
     </row>
     <row r="6" spans="1:19">
@@ -2232,7 +2185,7 @@
         <v>1</v>
       </c>
       <c r="R8" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="9" spans="1:19">
@@ -2338,7 +2291,7 @@
         <v>1</v>
       </c>
       <c r="R10" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="11" spans="1:19">
@@ -2444,7 +2397,7 @@
         <v>1</v>
       </c>
       <c r="R12" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -2497,7 +2450,7 @@
         <v>1</v>
       </c>
       <c r="R13" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="14" spans="1:19">
@@ -2550,7 +2503,7 @@
         <v>1</v>
       </c>
       <c r="R14" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="15" spans="1:19">
@@ -2706,7 +2659,7 @@
         <v>1</v>
       </c>
       <c r="R17" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="18" spans="1:19">
@@ -3021,7 +2974,7 @@
         <v>1</v>
       </c>
       <c r="S23" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="24" spans="1:19">

</xml_diff>